<commit_message>
MTTC and CI verified against Ozbay et al. (2008)
Read the original (TRR 2083, Eq. 2-7): the MTTC root selection and the
CI formula match the code exactly. Mass is left out as in the paper; the
paper's MTTC threshold is 4 s; CI = 0 when MTTC is inf follows the
paper's statement that constant-speed following gives CI = 0. Workbook
source cells (O37, J29) no longer say "unverified".

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SSM_dataset_metric_matrix.xlsx
+++ b/SSM_dataset_metric_matrix.xlsx
@@ -2651,6 +2651,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="37" t="inlineStr">
         <is>
@@ -4916,7 +4917,7 @@
       <c r="N37" s="42" t="inlineStr"/>
       <c r="O37" s="40" t="inlineStr">
         <is>
-          <t>Ozbay 等 2008（原文公式未核对）</t>
+          <t>Ozbay 等 2008（已对照原文 Eq. 7 核实）</t>
         </is>
       </c>
     </row>
@@ -5049,6 +5050,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="37" t="inlineStr">
         <is>
@@ -6345,7 +6347,7 @@
       </c>
       <c r="J29" s="40" t="inlineStr">
         <is>
-          <t>Ozbay 等 2008（原文公式未核对）</t>
+          <t>Ozbay 等 2008（已对照原文 Eq. 7 核实）</t>
         </is>
       </c>
     </row>
@@ -13629,8 +13631,8 @@
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="A1:W1"/>
     <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A34:D34"/>
     <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A34:D34"/>
     <mergeCell ref="A30:D30"/>
     <mergeCell ref="E2:L2"/>
     <mergeCell ref="M2:S2"/>

</xml_diff>